<commit_message>
v3.4.1 - Hilfe Screenshot-Galerie + Benutzeranleitung
- gui/hilfe_dialog.py: neuer Tab Vorschau (Screenshot-Kachelgalerie, Vollbild-Dialog, _ScreenshotCard, _FullscreenPreview)
- gui/main_window.py: grab_all_screenshots() - automatische PNG-Erstellung aller 14 Seiten
- docs/BENUTZERANLEITUNG.md: neue vollstaendige Benutzeranleitung (17 Abschnitte, Mockups, Diagramme)
- gui/mitarbeiter_dokumente.py: Tagesausweis-Panel (Bescheinigungen und Antraege)
- functions/mitarbeiter_dokumente_functions.py: Kategorie umbenannt
- config.py: APP_VERSION 3.4.1
- Alle MDs aktualisiert (v3.4.1)
</commit_message>
<xml_diff>
--- a/Daten/Sonderaufgaben/Sonderaufgaben.xlsx
+++ b/Daten/Sonderaufgaben/Sonderaufgaben.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="1076" documentId="13_ncr:1_{15C4A210-CED1-4F88-95AE-876D00722F5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A93D160-CB65-48A9-A17F-B9004B8C3F44}"/>
+  <xr:revisionPtr revIDLastSave="1080" documentId="13_ncr:1_{15C4A210-CED1-4F88-95AE-876D00722F5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52183854-22D8-454A-B67D-4FE47AB32069}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="21870" windowHeight="19550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43780" yWindow="1400" windowWidth="24440" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sonderaufgaben" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="38">
   <si>
     <t xml:space="preserve">    DRK KV Köln e.V. </t>
   </si>
@@ -145,18 +145,6 @@
   </si>
   <si>
     <t>Delgado</t>
-  </si>
-  <si>
-    <t>Köller</t>
-  </si>
-  <si>
-    <t>Heim</t>
-  </si>
-  <si>
-    <t>Touahni</t>
-  </si>
-  <si>
-    <t>Chugh</t>
   </si>
   <si>
     <t>Athanasiou</t>
@@ -783,10 +771,94 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -795,9 +867,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="7" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -823,87 +892,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1288,199 +1276,199 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="48.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="45" t="s">
+      <c r="B1" s="26"/>
+      <c r="C1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="46"/>
-      <c r="E1" s="47" t="s">
+      <c r="D1" s="28"/>
+      <c r="E1" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="48"/>
+      <c r="F1" s="30"/>
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="49">
+      <c r="A2" s="31">
         <f ca="1">TODAY()</f>
-        <v>46049</v>
-      </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="51" t="s">
+        <v>46092</v>
+      </c>
+      <c r="B2" s="32"/>
+      <c r="C2" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="52"/>
-      <c r="E2" s="51" t="s">
+      <c r="D2" s="34"/>
+      <c r="E2" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="34" t="s">
         <v>4</v>
       </c>
       <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7" ht="28.5" x14ac:dyDescent="0.65">
-      <c r="A3" s="53" t="s">
+      <c r="A3" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="55" t="s">
+      <c r="B3" s="36"/>
+      <c r="C3" s="37" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="56"/>
-      <c r="E3" s="55" t="s">
+      <c r="D3" s="38"/>
+      <c r="E3" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="56"/>
+      <c r="F3" s="38"/>
       <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" s="4" customFormat="1" ht="28.5" x14ac:dyDescent="0.65">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="55" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="56"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="16"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="42"/>
       <c r="G4" s="3"/>
     </row>
     <row r="5" spans="1:7" s="4" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="55" t="s">
+      <c r="B5" s="47"/>
+      <c r="C5" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="56"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="16"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="42"/>
       <c r="G5" s="3"/>
     </row>
     <row r="6" spans="1:7" ht="28.5" x14ac:dyDescent="0.65">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="16" t="s">
+      <c r="B6" s="40"/>
+      <c r="C6" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="16" t="s">
+      <c r="D6" s="43"/>
+      <c r="E6" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="17"/>
+      <c r="F6" s="43"/>
       <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" ht="28.5" x14ac:dyDescent="0.65">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="31"/>
-      <c r="C7" s="16" t="s">
+      <c r="B7" s="40"/>
+      <c r="C7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="17"/>
-      <c r="E7" s="32" t="s">
+      <c r="D7" s="43"/>
+      <c r="E7" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="33"/>
+      <c r="F7" s="45"/>
       <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" ht="28.5" x14ac:dyDescent="0.65">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="31"/>
-      <c r="C8" s="16" t="s">
+      <c r="B8" s="40"/>
+      <c r="C8" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="16" t="s">
+      <c r="D8" s="43"/>
+      <c r="E8" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="17"/>
+      <c r="F8" s="43"/>
       <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" ht="28.5" x14ac:dyDescent="0.65">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="16" t="s">
+      <c r="B9" s="40"/>
+      <c r="C9" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="32" t="s">
+      <c r="D9" s="43"/>
+      <c r="E9" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="F9" s="33"/>
+      <c r="F9" s="45"/>
       <c r="G9" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="28.5" x14ac:dyDescent="0.65">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="32" t="s">
+      <c r="B10" s="40"/>
+      <c r="C10" s="42" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="43"/>
+      <c r="E10" s="44" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="33"/>
+      <c r="F10" s="45"/>
       <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" s="4" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="36"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="18"/>
       <c r="G11" s="3"/>
     </row>
     <row r="12" spans="1:7" s="4" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="37"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="39"/>
+      <c r="A12" s="19"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="21"/>
       <c r="G12" s="3"/>
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="37"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="39"/>
+      <c r="A13" s="19"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="21"/>
       <c r="G13" s="3"/>
     </row>
     <row r="14" spans="1:7" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="40"/>
-      <c r="B14" s="41"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="42"/>
+      <c r="A14" s="22"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="24"/>
       <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" ht="28.5" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="51" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="25"/>
+      <c r="B15" s="52"/>
       <c r="C15" s="5" t="s">
         <v>16</v>
       </c>
@@ -1496,22 +1484,14 @@
       <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7" ht="28" x14ac:dyDescent="0.6">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>40</v>
-      </c>
+      <c r="B16" s="54"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
       <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
@@ -1521,12 +1501,12 @@
       <c r="B17" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="28" t="s">
+      <c r="C17" s="55"/>
+      <c r="D17" s="56"/>
+      <c r="E17" s="55" t="s">
         <v>22</v>
       </c>
-      <c r="F17" s="29"/>
+      <c r="F17" s="56"/>
       <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.4">
@@ -1536,16 +1516,16 @@
       <c r="B18" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="48">
         <v>44383</v>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="49">
         <v>43858</v>
       </c>
-      <c r="E18" s="23" t="s">
+      <c r="E18" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="F18" s="22"/>
+      <c r="F18" s="49"/>
     </row>
     <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="15"/>
@@ -1555,6 +1535,27 @@
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="C8:D8"/>
     <mergeCell ref="A11:F14"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
@@ -1571,27 +1572,6 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="75" orientation="landscape" r:id="rId1"/>

</xml_diff>